<commit_message>
Numera spools com 3 dígitos na relação do databook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBR97vd31m3ywVeV1zohhZ
</commit_message>
<xml_diff>
--- a/saida/Relacao_Databook_BRASNAVAL.xlsx
+++ b/saida/Relacao_Databook_BRASNAVAL.xlsx
@@ -553,7 +553,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-4012-Z02 / 01</t>
+          <t>24"-B1E-MR-4012-Z02 / 001</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-4012-Z02 / 02</t>
+          <t>24"-B1E-MR-4012-Z02 / 002</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-5003A-Z03 / 01</t>
+          <t>24"-B1E-MR-5003A-Z03 / 001</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-5003A-Z03 / 02</t>
+          <t>24"-B1E-MR-5003A-Z03 / 002</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-5003A-Z03 / 03</t>
+          <t>24"-B1E-MR-5003A-Z03 / 003</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-5003A-Z03 / 04</t>
+          <t>24"-B1E-MR-5003A-Z03 / 004</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 01</t>
+          <t>I-IS-025-421-510-46-9138 / 001</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -871,7 +871,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>MO7-4"-B3B-LO-5325A-PP-2 / 01</t>
+          <t>MO7-4"-B3B-LO-5325A-PP-2 / 001</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>6"-A1E-CF-4004A-Z02 / 01</t>
+          <t>6"-A1E-CF-4004A-Z02 / 001</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>8"-B3B-MR-4019A-Z02 / 01</t>
+          <t>8"-B3B-MR-4019A-Z02 / 001</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>8"-B3B-MR-4019A-Z02 / 02</t>
+          <t>8"-B3B-MR-4019A-Z02 / 002</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>4"-A3B-HF-4006A-Z03 / 01</t>
+          <t>4"-A3B-HF-4006A-Z03 / 001</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1073,7 +1073,7 @@
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 008; Spool não identificado no croqui – considerado spool único 01; Croqui: Extremidade com sobremetal</t>
+          <t>Mesmo desenho dos relatórios 008; Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidade com sobremetal</t>
         </is>
       </c>
     </row>
@@ -1101,7 +1101,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>4"-A3B-HF-4006A-Z03 / 01</t>
+          <t>4"-A3B-HF-4006A-Z03 / 001</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1119,7 +1119,7 @@
       </c>
       <c r="J14" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 007; Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Mesmo desenho dos relatórios 007; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2"-A1E-IA-911-Z03 / 01</t>
+          <t>2"-A1E-IA-911-Z03 / 001</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2"-A1E-IA-911-Z03 / 02</t>
+          <t>2"-A1E-IA-911-Z03 / 002</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9059 / 01</t>
+          <t>I-IS-025-421-510-46-9059 / 001</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>6"-D1E-NG-4301A-C-3"-Z02 / 01</t>
+          <t>6"-D1E-NG-4301A-C-3"-Z02 / 001</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>6"-D1E-NG-4301A-C-3"-Z02 / 02</t>
+          <t>6"-D1E-NG-4301A-C-3"-Z02 / 002</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 01</t>
+          <t>MO8-6"-B3B-MR-5405B-PP-2 / 001</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 030; Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Mesmo desenho dos relatórios 030; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>MO5-4"-B3B-LO-5119A-PP-2 / 01</t>
+          <t>MO5-4"-B3B-LO-5119A-PP-2 / 001</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9147 / 01</t>
+          <t>I-IS-025-421-510-46-9147 / 001</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
@@ -1479,7 +1479,7 @@
       </c>
       <c r="J22" s="4" t="inlineStr">
         <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 01; Croqui: Extremidades FT (solda de campo)</t>
+          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidades FT (solda de campo)</t>
         </is>
       </c>
     </row>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9148 / 01</t>
+          <t>I-IS-025-421-510-46-9148 / 001</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
@@ -1521,7 +1521,7 @@
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 01; Croqui: Extremidade FT (solda de campo)</t>
+          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidade FT (solda de campo)</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9150 / 01</t>
+          <t>I-IS-025-421-510-46-9150 / 001</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -1563,7 +1563,7 @@
       </c>
       <c r="J24" s="4" t="inlineStr">
         <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 01; Croqui idêntico ao do relatório 007; Croqui: Extremidade com sobremetal</t>
+          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui idêntico ao do relatório 007; Croqui: Extremidade com sobremetal</t>
         </is>
       </c>
     </row>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9151 / 01</t>
+          <t>I-IS-025-421-510-46-9151 / 001</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9160 / 01</t>
+          <t>I-IS-025-421-510-46-9160 / 001</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-9011 / 01</t>
+          <t>I-IS-025-421-510-9011 / 001</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="J27" s="4" t="inlineStr">
         <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 01; Croqui idêntico ao do relatório 008</t>
+          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui idêntico ao do relatório 008</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9165 / 01</t>
+          <t>I-IS-025-421-510-46-9165 / 001</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9165 / 02</t>
+          <t>I-IS-025-421-510-46-9165 / 002</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 01</t>
+          <t>I-IS-025-421-510-46-9138 / 001</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 02</t>
+          <t>I-IS-025-421-510-46-9138 / 002</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 03</t>
+          <t>I-IS-025-421-510-46-9138 / 003</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
@@ -1927,7 +1927,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 04</t>
+          <t>I-IS-025-421-510-46-9138 / 004</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>MO7-4"-B3B-LO-5309A-PP-2 / 01</t>
+          <t>MO7-4"-B3B-LO-5309A-PP-2 / 001</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>MO6-4"-B3B-LO-5113B-PP-2 / 01</t>
+          <t>MO6-4"-B3B-LO-5113B-PP-2 / 001</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2057,7 +2057,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>MO7-6"-B3B-MR-5405A-PP-2 / 01</t>
+          <t>MO7-6"-B3B-MR-5405A-PP-2 / 001</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2103,7 +2103,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>MO7-6"-B3B-MR-5405A-PP-2 / 02</t>
+          <t>MO7-6"-B3B-MR-5405A-PP-2 / 002</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2149,7 +2149,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>MO7-6"-B3B-MR-5405A-PP-2 / 03</t>
+          <t>MO7-6"-B3B-MR-5405A-PP-2 / 003</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>MO5-4"-B3B-MR-5113A-PP-2 / 01</t>
+          <t>MO5-4"-B3B-MR-5113A-PP-2 / 001</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2237,7 +2237,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 01</t>
+          <t>MO8-6"-B3B-MR-5405B-PP-2 / 001</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2283,7 +2283,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 02</t>
+          <t>MO8-6"-B3B-MR-5405B-PP-2 / 002</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2329,7 +2329,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 03</t>
+          <t>MO8-6"-B3B-MR-5405B-PP-2 / 003</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2375,7 +2375,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>MO5-10"-B3B-LO-5103A-2 / 01</t>
+          <t>MO5-10"-B3B-LO-5103A-2 / 001</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2421,7 +2421,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>MO5-10"-B3B-LO-5103A-2 / 02</t>
+          <t>MO5-10"-B3B-LO-5103A-2 / 002</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2467,7 +2467,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9067 / 01</t>
+          <t>I-IS-025-421-510-46-9067 / 001</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
@@ -2509,7 +2509,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9067 / 02</t>
+          <t>I-IS-025-421-510-46-9067 / 002</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
@@ -2551,7 +2551,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9067 / 03</t>
+          <t>I-IS-025-421-510-46-9067 / 003</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr"/>
@@ -2593,7 +2593,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9141 / 01</t>
+          <t>I-IS-025-421-510-46-9141 / 001</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
@@ -2635,7 +2635,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9141 / 02</t>
+          <t>I-IS-025-421-510-46-9141 / 002</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr"/>
@@ -2677,7 +2677,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 01</t>
+          <t>MO8-6"-B3B-MR-5405B-PP-2 / 001</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 02</t>
+          <t>MO8-6"-B3B-MR-5405B-PP-2 / 002</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -2769,7 +2769,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 03</t>
+          <t>MO8-6"-B3B-MR-5405B-PP-2 / 003</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -2815,7 +2815,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 04</t>
+          <t>MO8-6"-B3B-MR-5405B-PP-2 / 004</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -2861,7 +2861,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9048 / 01</t>
+          <t>I-IS-025-421-510-46-9048 / 001</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
@@ -2903,7 +2903,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9048 / 02</t>
+          <t>I-IS-025-421-510-46-9048 / 002</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr"/>
@@ -2945,7 +2945,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9048 / 03</t>
+          <t>I-IS-025-421-510-46-9048 / 003</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr"/>
@@ -2987,7 +2987,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9049 / 01</t>
+          <t>I-IS-025-421-510-46-9049 / 001</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr"/>
@@ -3029,7 +3029,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9049 / 02</t>
+          <t>I-IS-025-421-510-46-9049 / 002</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr"/>
@@ -3071,7 +3071,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9049 / 03</t>
+          <t>I-IS-025-421-510-46-9049 / 003</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr"/>
@@ -3113,7 +3113,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>6"-B3B-MR-5407A-PP-2 / 02</t>
+          <t>6"-B3B-MR-5407A-PP-2 / 002</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3159,7 +3159,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>6"-B3B-MR-5407A-PP-2 / 03</t>
+          <t>6"-B3B-MR-5407A-PP-2 / 003</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -3205,7 +3205,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9137 / 01</t>
+          <t>I-IS-025-421-510-46-9137 / 001</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr"/>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9137 / 02</t>
+          <t>I-IS-025-421-510-46-9137 / 002</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr"/>
@@ -3289,7 +3289,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9066 / 01</t>
+          <t>I-IS-025-421-510-46-9066 / 001</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
@@ -3331,7 +3331,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9066 / 02</t>
+          <t>I-IS-025-421-510-46-9066 / 002</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr"/>
@@ -3373,7 +3373,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9066 / 03</t>
+          <t>I-IS-025-421-510-46-9066 / 003</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
@@ -3415,7 +3415,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 01</t>
+          <t>I-IS-025-421-510-46-9138 / 001</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr"/>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 02</t>
+          <t>I-IS-025-421-510-46-9138 / 002</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr"/>
@@ -3499,7 +3499,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 03</t>
+          <t>I-IS-025-421-510-46-9138 / 003</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr"/>
@@ -3541,7 +3541,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 04</t>
+          <t>I-IS-025-421-510-46-9138 / 004</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr"/>
@@ -3687,7 +3687,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>01, 02</t>
+          <t>001, 002</t>
         </is>
       </c>
       <c r="H2" s="2" t="n">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03, 04</t>
+          <t>001, 002, 003, 004</t>
         </is>
       </c>
       <c r="H3" s="2" t="n">
@@ -3801,7 +3801,7 @@
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H5" s="2" t="n">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3919,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H6" s="2" t="n">
@@ -3978,7 +3978,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>01, 02</t>
+          <t>001, 002</t>
         </is>
       </c>
       <c r="H7" s="2" t="n">
@@ -4037,7 +4037,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
@@ -4061,7 +4061,7 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 008; Spool não identificado no croqui – considerado spool único 01; Croqui: Extremidade com sobremetal</t>
+          <t>Mesmo desenho dos relatórios 008; Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidade com sobremetal</t>
         </is>
       </c>
     </row>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
@@ -4120,7 +4120,7 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 007; Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Mesmo desenho dos relatórios 007; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4155,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>01, 02</t>
+          <t>001, 002</t>
         </is>
       </c>
       <c r="H10" s="2" t="n">
@@ -4210,7 +4210,7 @@
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -4269,7 +4269,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>01, 02</t>
+          <t>001, 002</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H13" s="2" t="n">
@@ -4352,7 +4352,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 030; Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Mesmo desenho dos relatórios 030; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H14" s="2" t="n">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -4442,7 +4442,7 @@
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
@@ -4466,7 +4466,7 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 01; Croqui: Extremidades FT (solda de campo)</t>
+          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidades FT (solda de campo)</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4497,7 @@
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
@@ -4521,7 +4521,7 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 01; Croqui: Extremidade FT (solda de campo)</t>
+          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui: Extremidade FT (solda de campo)</t>
         </is>
       </c>
     </row>
@@ -4552,7 +4552,7 @@
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H17" s="2" t="n">
@@ -4576,7 +4576,7 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 01; Croqui idêntico ao do relatório 007; Croqui: Extremidade com sobremetal</t>
+          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui idêntico ao do relatório 007; Croqui: Extremidade com sobremetal</t>
         </is>
       </c>
     </row>
@@ -4607,7 +4607,7 @@
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -4662,7 +4662,7 @@
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H19" s="2" t="n">
@@ -4717,7 +4717,7 @@
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H20" s="2" t="n">
@@ -4741,7 +4741,7 @@
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 01; Croqui idêntico ao do relatório 008</t>
+          <t>TAG não consta no relatório (referência é o isométrico); Spool não identificado no croqui – considerado spool único 001; Croqui idêntico ao do relatório 008</t>
         </is>
       </c>
     </row>
@@ -4772,7 +4772,7 @@
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>01, 02</t>
+          <t>001, 002</t>
         </is>
       </c>
       <c r="H21" s="2" t="n">
@@ -4827,7 +4827,7 @@
       <c r="F22" s="2" t="inlineStr"/>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03, 04</t>
+          <t>001, 002, 003, 004</t>
         </is>
       </c>
       <c r="H22" s="2" t="n">
@@ -4886,7 +4886,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H23" s="2" t="n">
@@ -4910,7 +4910,7 @@
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 01</t>
+          <t>Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -4945,7 +4945,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H24" s="2" t="n">
@@ -5000,7 +5000,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03</t>
+          <t>001, 002, 003</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>01</t>
+          <t>001</t>
         </is>
       </c>
       <c r="H26" s="2" t="n">
@@ -5114,7 +5114,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03</t>
+          <t>001, 002, 003</t>
         </is>
       </c>
       <c r="H27" s="2" t="n">
@@ -5173,7 +5173,7 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>01, 02</t>
+          <t>001, 002</t>
         </is>
       </c>
       <c r="H28" s="2" t="n">
@@ -5228,7 +5228,7 @@
       <c r="F29" s="2" t="inlineStr"/>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03</t>
+          <t>001, 002, 003</t>
         </is>
       </c>
       <c r="H29" s="2" t="n">
@@ -5283,7 +5283,7 @@
       <c r="F30" s="2" t="inlineStr"/>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>01, 02</t>
+          <t>001, 002</t>
         </is>
       </c>
       <c r="H30" s="2" t="n">
@@ -5342,7 +5342,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03, 04</t>
+          <t>001, 002, 003, 004</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">
@@ -5397,7 +5397,7 @@
       <c r="F32" s="2" t="inlineStr"/>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03</t>
+          <t>001, 002, 003</t>
         </is>
       </c>
       <c r="H32" s="2" t="n">
@@ -5452,7 +5452,7 @@
       <c r="F33" s="2" t="inlineStr"/>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03</t>
+          <t>001, 002, 003</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
@@ -5511,7 +5511,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>02, 03</t>
+          <t>002, 003</t>
         </is>
       </c>
       <c r="H34" s="2" t="n">
@@ -5566,7 +5566,7 @@
       <c r="F35" s="2" t="inlineStr"/>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>01, 02</t>
+          <t>001, 002</t>
         </is>
       </c>
       <c r="H35" s="2" t="n">
@@ -5621,7 +5621,7 @@
       <c r="F36" s="2" t="inlineStr"/>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03</t>
+          <t>001, 002, 003</t>
         </is>
       </c>
       <c r="H36" s="2" t="n">
@@ -5676,7 +5676,7 @@
       <c r="F37" s="2" t="inlineStr"/>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>01, 02, 03, 04</t>
+          <t>001, 002, 003, 004</t>
         </is>
       </c>
       <c r="H37" s="2" t="n">

</xml_diff>

<commit_message>
Spool só com o número e coluna TAG PADRONIZADA no databook
A coluna Spool passa a ter apenas o nº (001, 002...). A TAG da linha vira
TAG PADRONIZADA (DN-CLASS-SERVICE-LINE_NUMBER, 4 blocos), com prefixo de
módulo MOx removido e observação quando não há TAG no relatório.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YBR97vd31m3ywVeV1zohhZ
</commit_message>
<xml_diff>
--- a/saida/Relacao_Databook_BRASNAVAL.xlsx
+++ b/saida/Relacao_Databook_BRASNAVAL.xlsx
@@ -470,7 +470,7 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="40" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
@@ -510,7 +510,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>TAG da linha</t>
+          <t>TAG PADRONIZADA</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -553,7 +553,7 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-4012-Z02 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -599,7 +599,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-4012-Z02 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-5003A-Z03 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -691,7 +691,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-5003A-Z03 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -737,7 +737,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-5003A-Z03 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -783,7 +783,7 @@
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>24"-B1E-MR-5003A-Z03 / 004</t>
+          <t>004</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
@@ -829,7 +829,7 @@
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr"/>
@@ -871,7 +871,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>MO7-4"-B3B-LO-5325A-PP-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 001</t>
+          <t>Prefixo de módulo MO7 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>6"-A1E-CF-4004A-Z02 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>8"-B3B-MR-4019A-Z02 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -1009,7 +1009,7 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>8"-B3B-MR-4019A-Z02 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1055,7 +1055,7 @@
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>4"-A3B-HF-4006A-Z03 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
@@ -1101,7 +1101,7 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>4"-A3B-HF-4006A-Z03 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>2"-A1E-IA-911-Z03 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>2"-A1E-IA-911-Z03 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
@@ -1239,7 +1239,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9059 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr"/>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>6"-D1E-NG-4301A-C-3"-Z02 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -1327,7 +1327,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>6"-D1E-NG-4301A-C-3"-Z02 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
@@ -1391,7 +1391,7 @@
       </c>
       <c r="J20" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 030; Spool não identificado no croqui – considerado spool único 001</t>
+          <t>Mesmo desenho dos relatórios 030; Prefixo de módulo MO8 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -1419,7 +1419,7 @@
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>MO5-4"-B3B-LO-5119A-PP-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="J21" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 001</t>
+          <t>Prefixo de módulo MO5 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1465,7 @@
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9147 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr"/>
@@ -1507,7 +1507,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9148 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr"/>
@@ -1549,7 +1549,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9150 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr"/>
@@ -1591,7 +1591,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9151 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr"/>
@@ -1633,7 +1633,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9160 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr"/>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-9011 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr"/>
@@ -1717,7 +1717,7 @@
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9165 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr"/>
@@ -1759,7 +1759,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9165 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr"/>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr"/>
@@ -1843,7 +1843,7 @@
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr"/>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr"/>
@@ -1927,7 +1927,7 @@
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 004</t>
+          <t>004</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr"/>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>MO7-4"-B3B-LO-5309A-PP-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
@@ -1987,7 +1987,7 @@
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 001</t>
+          <t>Prefixo de módulo MO7 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>MO6-4"-B3B-LO-5113B-PP-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2031,7 +2031,11 @@
       <c r="I35" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="J35" s="2" t="inlineStr"/>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo de módulo MO6 removido</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2057,7 +2061,7 @@
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>MO7-6"-B3B-MR-5405A-PP-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
@@ -2075,7 +2079,7 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido nas juntas 06 e 20</t>
+          <t>Prefixo de módulo MO7 removido; Croqui: Spool dividido nas juntas 06 e 20</t>
         </is>
       </c>
     </row>
@@ -2103,7 +2107,7 @@
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>MO7-6"-B3B-MR-5405A-PP-2 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
@@ -2121,7 +2125,7 @@
       </c>
       <c r="J37" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido nas juntas 06 e 20</t>
+          <t>Prefixo de módulo MO7 removido; Croqui: Spool dividido nas juntas 06 e 20</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2153,7 @@
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>MO7-6"-B3B-MR-5405A-PP-2 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -2167,7 +2171,7 @@
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido nas juntas 06 e 20</t>
+          <t>Prefixo de módulo MO7 removido; Croqui: Spool dividido nas juntas 06 e 20</t>
         </is>
       </c>
     </row>
@@ -2195,7 +2199,7 @@
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>MO5-4"-B3B-MR-5113A-PP-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
@@ -2211,7 +2215,11 @@
       <c r="I39" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="J39" s="2" t="inlineStr"/>
+      <c r="J39" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo de módulo MO5 removido</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2237,7 +2245,7 @@
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
@@ -2255,7 +2263,7 @@
       </c>
       <c r="J40" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido nas juntas 04 e 12</t>
+          <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 04 e 12</t>
         </is>
       </c>
     </row>
@@ -2283,7 +2291,7 @@
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
@@ -2301,7 +2309,7 @@
       </c>
       <c r="J41" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido nas juntas 04 e 12</t>
+          <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 04 e 12</t>
         </is>
       </c>
     </row>
@@ -2329,7 +2337,7 @@
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -2347,7 +2355,7 @@
       </c>
       <c r="J42" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido nas juntas 04 e 12</t>
+          <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 04 e 12</t>
         </is>
       </c>
     </row>
@@ -2375,7 +2383,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>MO5-10"-B3B-LO-5103A-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2393,7 +2401,7 @@
       </c>
       <c r="J43" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido na junta 04</t>
+          <t>Prefixo de módulo MO5 removido; Croqui: Spool dividido na junta 04</t>
         </is>
       </c>
     </row>
@@ -2421,7 +2429,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>MO5-10"-B3B-LO-5103A-2 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2439,7 +2447,7 @@
       </c>
       <c r="J44" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido na junta 04</t>
+          <t>Prefixo de módulo MO5 removido; Croqui: Spool dividido na junta 04</t>
         </is>
       </c>
     </row>
@@ -2467,7 +2475,7 @@
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9067 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G45" s="2" t="inlineStr"/>
@@ -2509,7 +2517,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9067 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G46" s="2" t="inlineStr"/>
@@ -2551,7 +2559,7 @@
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9067 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr"/>
@@ -2593,7 +2601,7 @@
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9141 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr"/>
@@ -2635,7 +2643,7 @@
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9141 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr"/>
@@ -2677,7 +2685,7 @@
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G50" s="2" t="inlineStr">
@@ -2695,7 +2703,7 @@
       </c>
       <c r="J50" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 012; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+          <t>Mesmo desenho dos relatórios 012; Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
         </is>
       </c>
     </row>
@@ -2723,7 +2731,7 @@
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G51" s="2" t="inlineStr">
@@ -2741,7 +2749,7 @@
       </c>
       <c r="J51" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 012; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+          <t>Mesmo desenho dos relatórios 012; Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2777,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -2787,7 +2795,7 @@
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 012; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+          <t>Mesmo desenho dos relatórios 012; Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
         </is>
       </c>
     </row>
@@ -2815,7 +2823,7 @@
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
-          <t>MO8-6"-B3B-MR-5405B-PP-2 / 004</t>
+          <t>004</t>
         </is>
       </c>
       <c r="G53" s="2" t="inlineStr">
@@ -2833,7 +2841,7 @@
       </c>
       <c r="J53" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 012; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+          <t>Mesmo desenho dos relatórios 012; Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
         </is>
       </c>
     </row>
@@ -2861,7 +2869,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9048 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr"/>
@@ -2903,7 +2911,7 @@
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9048 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr"/>
@@ -2945,7 +2953,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9048 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr"/>
@@ -2987,7 +2995,7 @@
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9049 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr"/>
@@ -3029,7 +3037,7 @@
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9049 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr"/>
@@ -3071,7 +3079,7 @@
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9049 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G59" s="2" t="inlineStr"/>
@@ -3113,7 +3121,7 @@
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
-          <t>6"-B3B-MR-5407A-PP-2 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G60" s="2" t="inlineStr">
@@ -3159,7 +3167,7 @@
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
-          <t>6"-B3B-MR-5407A-PP-2 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G61" s="2" t="inlineStr">
@@ -3205,7 +3213,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9137 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr"/>
@@ -3247,7 +3255,7 @@
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9137 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G63" s="2" t="inlineStr"/>
@@ -3289,7 +3297,7 @@
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9066 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G64" s="2" t="inlineStr"/>
@@ -3331,7 +3339,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9066 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr"/>
@@ -3373,7 +3381,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9066 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr"/>
@@ -3415,7 +3423,7 @@
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 001</t>
+          <t>001</t>
         </is>
       </c>
       <c r="G67" s="2" t="inlineStr"/>
@@ -3457,7 +3465,7 @@
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 002</t>
+          <t>002</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr"/>
@@ -3499,7 +3507,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 003</t>
+          <t>003</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr"/>
@@ -3541,7 +3549,7 @@
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>I-IS-025-421-510-46-9138 / 004</t>
+          <t>004</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr"/>
@@ -3617,7 +3625,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>TAG da linha</t>
+          <t>TAG PADRONIZADA</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -3884,7 +3892,7 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 001</t>
+          <t>Prefixo de módulo MO7 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -4352,7 +4360,7 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 030; Spool não identificado no croqui – considerado spool único 001</t>
+          <t>Mesmo desenho dos relatórios 030; Prefixo de módulo MO8 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4419,7 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 001</t>
+          <t>Prefixo de módulo MO5 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4918,7 @@
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>Spool não identificado no croqui – considerado spool único 001</t>
+          <t>Prefixo de módulo MO7 removido; Spool não identificado no croqui – considerado spool único 001</t>
         </is>
       </c>
     </row>
@@ -4967,7 +4975,11 @@
       <c r="L24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo de módulo MO6 removido</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -5024,7 +5036,7 @@
       </c>
       <c r="M25" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido nas juntas 06 e 20</t>
+          <t>Prefixo de módulo MO7 removido; Croqui: Spool dividido nas juntas 06 e 20</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5093,11 @@
       <c r="L26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>Prefixo de módulo MO5 removido</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -5138,7 +5154,7 @@
       </c>
       <c r="M27" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido nas juntas 04 e 12</t>
+          <t>Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 04 e 12</t>
         </is>
       </c>
     </row>
@@ -5197,7 +5213,7 @@
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>Croqui: Spool dividido na junta 04</t>
+          <t>Prefixo de módulo MO5 removido; Croqui: Spool dividido na junta 04</t>
         </is>
       </c>
     </row>
@@ -5366,7 +5382,7 @@
       </c>
       <c r="M31" s="4" t="inlineStr">
         <is>
-          <t>Mesmo desenho dos relatórios 012; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
+          <t>Mesmo desenho dos relatórios 012; Prefixo de módulo MO8 removido; Croqui: Spool dividido nas juntas 08, 16 e 28</t>
         </is>
       </c>
     </row>
@@ -5743,7 +5759,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>TAG da linha</t>
+          <t>TAG PADRONIZADA</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">

</xml_diff>